<commit_message>
cleansing and slide 8
</commit_message>
<xml_diff>
--- a/testing.xlsx
+++ b/testing.xlsx
@@ -8,27 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\renato\projetos\double-projects\ppt-doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9697AFE-67AF-4EF7-86F2-C22B8F53708D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071CF139-2C15-49A9-81E8-22D83EEBF4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="5" xr2:uid="{E2EAAA9B-09FC-4773-92F8-622FD93420C8}"/>
+    <workbookView xWindow="1875" yWindow="1425" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{E2EAAA9B-09FC-4773-92F8-622FD93420C8}"/>
   </bookViews>
   <sheets>
-    <sheet name="DRE Saida" sheetId="1" r:id="rId1"/>
-    <sheet name="Pizza Teste" sheetId="6" r:id="rId2"/>
-    <sheet name="slide_8" sheetId="7" r:id="rId3"/>
-    <sheet name="slide_9" sheetId="8" r:id="rId4"/>
-    <sheet name="slide_11" sheetId="9" r:id="rId5"/>
-    <sheet name="Carteira" sheetId="16" r:id="rId6"/>
-    <sheet name="slide_12" sheetId="10" r:id="rId7"/>
-    <sheet name="slide_13" sheetId="11" r:id="rId8"/>
-    <sheet name="slide_14" sheetId="12" r:id="rId9"/>
-    <sheet name="slide_15" sheetId="13" r:id="rId10"/>
-    <sheet name="slide_18" sheetId="14" r:id="rId11"/>
-    <sheet name="slide_20" sheetId="15" r:id="rId12"/>
-    <sheet name="Qualidade Cart 2682" sheetId="3" r:id="rId13"/>
-    <sheet name="Emprestimos" sheetId="4" r:id="rId14"/>
-    <sheet name="Seguros e Cartoes" sheetId="5" r:id="rId15"/>
-    <sheet name="Margem Financeira" sheetId="2" r:id="rId16"/>
+    <sheet name="DRE Saida 2" sheetId="18" r:id="rId1"/>
+    <sheet name="Tabelas" sheetId="19" r:id="rId2"/>
+    <sheet name="DRE Saida" sheetId="1" r:id="rId3"/>
+    <sheet name="Pizza Teste" sheetId="6" r:id="rId4"/>
+    <sheet name="slide_8" sheetId="7" r:id="rId5"/>
+    <sheet name="slide_9" sheetId="8" r:id="rId6"/>
+    <sheet name="slide_11" sheetId="9" r:id="rId7"/>
+    <sheet name="Carteira" sheetId="16" r:id="rId8"/>
+    <sheet name="slide_12" sheetId="10" r:id="rId9"/>
+    <sheet name="slide_13" sheetId="11" r:id="rId10"/>
+    <sheet name="slide_14" sheetId="12" r:id="rId11"/>
+    <sheet name="slide_15" sheetId="13" r:id="rId12"/>
+    <sheet name="slide_18" sheetId="14" r:id="rId13"/>
+    <sheet name="slide_20" sheetId="15" r:id="rId14"/>
+    <sheet name="Qualidade Cart 2682" sheetId="3" r:id="rId15"/>
+    <sheet name="Emprestimos" sheetId="4" r:id="rId16"/>
+    <sheet name="Seguros e Cartoes" sheetId="5" r:id="rId17"/>
+    <sheet name="Margem Financeira" sheetId="2" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="143">
   <si>
     <t>Labels</t>
   </si>
@@ -465,6 +467,24 @@
   </si>
   <si>
     <t>TVM privado</t>
+  </si>
+  <si>
+    <t>Receita de Prestação de Serviços e Corretagem</t>
+  </si>
+  <si>
+    <t>Margem Financeira Com Clientes</t>
+  </si>
+  <si>
+    <t>Margem Financeira com Mercado</t>
+  </si>
+  <si>
+    <t>Receitas de Corretagem e Seguro</t>
+  </si>
+  <si>
+    <t>Receitas de Prestação de Servicos e Corretagem</t>
+  </si>
+  <si>
+    <t>Receitas de Prestação de Serviços (exclui corretagem de seguros)</t>
   </si>
 </sst>
 </file>
@@ -534,7 +554,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -556,6 +576,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -890,169 +911,167 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{417E299C-E79D-4FD4-B55D-DB1E7B3327CE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D0A736-06AB-48E7-AFFE-0EC2903148F5}">
   <dimension ref="B3:N36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="42.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1</v>
-      </c>
+    <row r="3" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18">
-        <v>285</v>
-      </c>
-      <c r="D18">
-        <v>302</v>
-      </c>
-      <c r="E18">
-        <v>321</v>
-      </c>
-      <c r="F18">
-        <v>363</v>
-      </c>
-      <c r="G18">
-        <v>496</v>
-      </c>
-      <c r="H18">
-        <v>542</v>
-      </c>
-      <c r="I18">
-        <v>480</v>
-      </c>
-      <c r="J18">
-        <v>459</v>
-      </c>
-      <c r="K18">
-        <v>461</v>
-      </c>
-      <c r="L18">
-        <v>1180</v>
-      </c>
-      <c r="M18">
-        <v>1400</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="G3">
+        <v>2024</v>
+      </c>
+      <c r="H3">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="4" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4">
+        <v>3214</v>
+      </c>
+      <c r="E4">
+        <v>2919</v>
+      </c>
+      <c r="F4">
+        <v>3136</v>
+      </c>
+      <c r="G4">
+        <v>11980</v>
+      </c>
+      <c r="H4">
+        <v>11913</v>
+      </c>
+    </row>
+    <row r="5" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5">
+        <v>2519</v>
+      </c>
+      <c r="E5">
+        <v>2295</v>
+      </c>
+      <c r="F5">
+        <v>2304</v>
+      </c>
+      <c r="G5">
+        <v>9301</v>
+      </c>
+      <c r="H5">
+        <v>9283</v>
+      </c>
+    </row>
+    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6">
+        <v>2367</v>
+      </c>
+      <c r="E6">
+        <v>2051</v>
+      </c>
+      <c r="F6">
+        <v>2131</v>
+      </c>
+      <c r="G6">
+        <v>8353</v>
+      </c>
+      <c r="H6">
+        <v>8317</v>
+      </c>
+    </row>
+    <row r="7" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7">
+        <v>152</v>
+      </c>
+      <c r="E7">
+        <v>244</v>
+      </c>
+      <c r="F7">
+        <v>172</v>
+      </c>
+      <c r="G7">
+        <v>947</v>
+      </c>
+      <c r="H7">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="9" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9">
+        <v>695</v>
+      </c>
+      <c r="E9">
+        <v>624</v>
+      </c>
+      <c r="F9">
+        <v>832</v>
+      </c>
+      <c r="G9">
+        <v>2679</v>
+      </c>
+      <c r="H9">
+        <v>2630</v>
+      </c>
+    </row>
+    <row r="18" spans="3:14" x14ac:dyDescent="0.25">
       <c r="N18" s="1"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="C20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="L20" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+    </row>
+    <row r="21" spans="3:14" x14ac:dyDescent="0.25">
       <c r="L21" s="1"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="C25" s="4">
-        <v>0.09</v>
-      </c>
-      <c r="D25" s="5">
-        <v>9.4E-2</v>
-      </c>
-      <c r="E25" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="F25" s="5">
-        <v>0.111</v>
-      </c>
-      <c r="G25" s="4">
-        <v>0.15</v>
-      </c>
-      <c r="H25" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="I25" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="J25" s="5">
-        <v>0.151</v>
-      </c>
-      <c r="K25" s="4">
-        <v>0.15</v>
-      </c>
-      <c r="L25" s="5">
-        <v>0.121</v>
-      </c>
-      <c r="M25" s="5">
-        <v>0.154</v>
-      </c>
+    <row r="25" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C25" s="4"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="B35" s="2"/>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B36" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1061,6 +1080,264 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC81BA9-A722-4D51-8849-833605DBA551}">
+  <dimension ref="B4:O7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B4" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="J4" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="13"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" t="s">
+        <v>5</v>
+      </c>
+      <c r="L5" t="s">
+        <v>8</v>
+      </c>
+      <c r="M5" t="s">
+        <v>9</v>
+      </c>
+      <c r="N5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D6" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="E6" s="10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F6" s="10">
+        <v>3.1</v>
+      </c>
+      <c r="G6" s="10">
+        <v>3</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="K6" s="3">
+        <v>0.41</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0.41</v>
+      </c>
+      <c r="M6" s="3">
+        <v>0.41</v>
+      </c>
+      <c r="N6" s="3">
+        <v>0.42</v>
+      </c>
+      <c r="O6" s="3">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="12">
+        <v>6.4</v>
+      </c>
+      <c r="D7" s="12">
+        <v>4.7</v>
+      </c>
+      <c r="E7" s="12">
+        <v>5.4</v>
+      </c>
+      <c r="F7" s="12">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="G7" s="12">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="J4:O4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB40F4D6-7254-451B-8F15-55583AC6E46C}">
+  <dimension ref="B2:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3">
+        <v>5.5</v>
+      </c>
+      <c r="D3">
+        <v>1.3</v>
+      </c>
+      <c r="E3">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4">
+        <v>6.5</v>
+      </c>
+      <c r="D4">
+        <v>5.3</v>
+      </c>
+      <c r="E4">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5">
+        <v>37.1</v>
+      </c>
+      <c r="D5">
+        <v>28.4</v>
+      </c>
+      <c r="E5">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6">
+        <v>3.2</v>
+      </c>
+      <c r="D6">
+        <v>3.4</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7">
+        <v>10.4</v>
+      </c>
+      <c r="D7">
+        <v>6.8</v>
+      </c>
+      <c r="E7">
+        <v>8.8000000000000007</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8">
+        <v>0.7</v>
+      </c>
+      <c r="D8">
+        <v>0.8</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9">
+        <v>4.2</v>
+      </c>
+      <c r="D9">
+        <v>7.2</v>
+      </c>
+      <c r="E9">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10">
+        <v>35</v>
+      </c>
+      <c r="D10">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="E10">
+        <v>41.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53DDA400-E7C3-412D-BF6F-6237B27DC1D6}">
   <dimension ref="D2:O7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1209,7 +1486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2216C394-E57F-4E0F-A385-35E21DA9536A}">
   <dimension ref="A3:N5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1294,7 +1571,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C78759-C237-4426-A1F9-93877BD87587}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1590,7 +1867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61B4CFF7-3A85-4820-951F-62E41E9FBB53}">
   <dimension ref="B7:P10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1788,7 +2065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E23628D-2121-49A9-92D5-277D45F162FD}">
   <dimension ref="C4:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1926,7 +2203,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F3A3B47-E08A-478E-9E32-E383F8DD5BE7}">
   <dimension ref="C14:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1964,7 +2241,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB80353-2AEA-4B03-BD7E-AB8ECF39D507}">
   <dimension ref="W3:AK9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2045,6 +2322,273 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2DB3A40-3823-4B44-8654-968315449624}">
+  <dimension ref="C16:H31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="59.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="16" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>121</v>
+      </c>
+      <c r="G16">
+        <v>2024</v>
+      </c>
+      <c r="H16">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H17" s="15"/>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D19">
+        <v>239</v>
+      </c>
+      <c r="E19">
+        <v>205</v>
+      </c>
+      <c r="F19">
+        <v>290</v>
+      </c>
+      <c r="G19">
+        <v>932</v>
+      </c>
+      <c r="H19">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>141</v>
+      </c>
+      <c r="D26">
+        <v>695</v>
+      </c>
+      <c r="E26">
+        <v>624</v>
+      </c>
+      <c r="F26">
+        <v>832</v>
+      </c>
+      <c r="G26">
+        <v>2679</v>
+      </c>
+      <c r="H26">
+        <v>2630</v>
+      </c>
+    </row>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28">
+        <v>457</v>
+      </c>
+      <c r="E28">
+        <v>419</v>
+      </c>
+      <c r="F28">
+        <v>542</v>
+      </c>
+      <c r="G28">
+        <v>1748</v>
+      </c>
+      <c r="H28">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="F31" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{417E299C-E79D-4FD4-B55D-DB1E7B3327CE}">
+  <dimension ref="B3:N36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18">
+        <v>285</v>
+      </c>
+      <c r="D18">
+        <v>302</v>
+      </c>
+      <c r="E18">
+        <v>321</v>
+      </c>
+      <c r="F18">
+        <v>363</v>
+      </c>
+      <c r="G18">
+        <v>496</v>
+      </c>
+      <c r="H18">
+        <v>542</v>
+      </c>
+      <c r="I18">
+        <v>480</v>
+      </c>
+      <c r="J18">
+        <v>459</v>
+      </c>
+      <c r="K18">
+        <v>461</v>
+      </c>
+      <c r="L18">
+        <v>1180</v>
+      </c>
+      <c r="M18">
+        <v>1400</v>
+      </c>
+      <c r="N18" s="1"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="L21" s="1"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C25" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="D25" s="5">
+        <v>9.4E-2</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="F25" s="5">
+        <v>0.111</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="H25" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="I25" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="J25" s="5">
+        <v>0.151</v>
+      </c>
+      <c r="K25" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="L25" s="5">
+        <v>0.121</v>
+      </c>
+      <c r="M25" s="5">
+        <v>0.154</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44452379-0FE0-41DB-BDE4-79B6F1D7D785}">
   <dimension ref="A1:N285"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3903,7 +4447,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23508980-3939-4D95-9A4C-23A64D6BD062}">
   <dimension ref="C3:J27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4145,7 +4689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64FAFF65-4D1E-443F-BDF3-D7DA42FEA733}">
   <dimension ref="B2:P7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4287,7 +4831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B33BFE8-86C2-496F-B733-78BC5607B7C2}">
   <dimension ref="B2:O6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4437,7 +4981,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3790767E-187D-4BED-BBAB-0D1EEC80F334}">
   <dimension ref="C12:N36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4733,7 +5277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4745116-4A8C-412D-BBE6-45B5E5EC0DB3}">
   <dimension ref="B3:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4867,262 +5411,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC81BA9-A722-4D51-8849-833605DBA551}">
-  <dimension ref="B4:O7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="J4" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>12</v>
-      </c>
-      <c r="K5" t="s">
-        <v>5</v>
-      </c>
-      <c r="L5" t="s">
-        <v>8</v>
-      </c>
-      <c r="M5" t="s">
-        <v>9</v>
-      </c>
-      <c r="N5" t="s">
-        <v>11</v>
-      </c>
-      <c r="O5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="10">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.9</v>
-      </c>
-      <c r="E6" s="10">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F6" s="10">
-        <v>3.1</v>
-      </c>
-      <c r="G6" s="10">
-        <v>3</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="K6" s="3">
-        <v>0.41</v>
-      </c>
-      <c r="L6" s="3">
-        <v>0.41</v>
-      </c>
-      <c r="M6" s="3">
-        <v>0.41</v>
-      </c>
-      <c r="N6" s="3">
-        <v>0.42</v>
-      </c>
-      <c r="O6" s="3">
-        <v>0.41</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="12">
-        <v>6.4</v>
-      </c>
-      <c r="D7" s="12">
-        <v>4.7</v>
-      </c>
-      <c r="E7" s="12">
-        <v>5.4</v>
-      </c>
-      <c r="F7" s="12">
-        <v>18.100000000000001</v>
-      </c>
-      <c r="G7" s="12">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="J4:O4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB40F4D6-7254-451B-8F15-55583AC6E46C}">
-  <dimension ref="B2:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3">
-        <v>5.5</v>
-      </c>
-      <c r="D3">
-        <v>1.3</v>
-      </c>
-      <c r="E3">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4">
-        <v>6.5</v>
-      </c>
-      <c r="D4">
-        <v>5.3</v>
-      </c>
-      <c r="E4">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5">
-        <v>37.1</v>
-      </c>
-      <c r="D5">
-        <v>28.4</v>
-      </c>
-      <c r="E5">
-        <v>30.4</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6">
-        <v>3.2</v>
-      </c>
-      <c r="D6">
-        <v>3.4</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7">
-        <v>10.4</v>
-      </c>
-      <c r="D7">
-        <v>6.8</v>
-      </c>
-      <c r="E7">
-        <v>8.8000000000000007</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8">
-        <v>0.7</v>
-      </c>
-      <c r="D8">
-        <v>0.8</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9">
-        <v>4.2</v>
-      </c>
-      <c r="D9">
-        <v>7.2</v>
-      </c>
-      <c r="E9">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10">
-        <v>35</v>
-      </c>
-      <c r="D10">
-        <v>40.799999999999997</v>
-      </c>
-      <c r="E10">
-        <v>41.9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fine tuning no slide 21
</commit_message>
<xml_diff>
--- a/testing.xlsx
+++ b/testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\renato\projetos\double-projects\ppt-doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B88A98-8B26-43E9-83A4-B36059BA0ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01012DF-D5F2-417F-8986-A07C75BC6E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="901" activeTab="6" xr2:uid="{E2EAAA9B-09FC-4773-92F8-622FD93420C8}"/>
   </bookViews>
@@ -4493,10 +4493,10 @@
         <v>105</v>
       </c>
       <c r="D4" s="8">
-        <v>0.01</v>
+        <v>0.12</v>
       </c>
       <c r="F4" s="8">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -4504,10 +4504,10 @@
         <v>106</v>
       </c>
       <c r="D5" s="8">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
       <c r="F5" s="8">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -4515,10 +4515,10 @@
         <v>107</v>
       </c>
       <c r="D6" s="8">
-        <v>0.03</v>
+        <v>0.1</v>
       </c>
       <c r="F6" s="8">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -4526,10 +4526,10 @@
         <v>108</v>
       </c>
       <c r="D7" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="F7" s="8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -4537,10 +4537,10 @@
         <v>109</v>
       </c>
       <c r="D8" s="8">
-        <v>0.06</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F8" s="8">
-        <v>0.01</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -4548,10 +4548,10 @@
         <v>110</v>
       </c>
       <c r="D9" s="8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F9" s="8">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -4559,7 +4559,7 @@
         <v>111</v>
       </c>
       <c r="D10" s="8">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="F10" s="8">
         <v>0.05</v>
@@ -4570,10 +4570,10 @@
         <v>112</v>
       </c>
       <c r="D11" s="8">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
       <c r="F11" s="8">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>0.04</v>
       </c>
       <c r="F12" s="8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -4592,10 +4592,10 @@
         <v>114</v>
       </c>
       <c r="D13" s="8">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="F13" s="8">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -4603,10 +4603,10 @@
         <v>115</v>
       </c>
       <c r="D14" s="8">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="F14" s="8">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -4614,10 +4614,10 @@
         <v>116</v>
       </c>
       <c r="D15" s="8">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="F15" s="8">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -4625,10 +4625,10 @@
         <v>117</v>
       </c>
       <c r="D16" s="8">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="F16" s="8">
-        <v>0.09</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -4636,10 +4636,10 @@
         <v>118</v>
       </c>
       <c r="D17" s="8">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="F17" s="8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -4647,7 +4647,7 @@
         <v>119</v>
       </c>
       <c r="D18" s="8">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="F18" s="8">
         <v>0.02</v>
@@ -4658,10 +4658,10 @@
         <v>120</v>
       </c>
       <c r="D19" s="8">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="F19" s="8">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -4669,10 +4669,10 @@
         <v>121</v>
       </c>
       <c r="D20" s="8">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="F20" s="8">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -4680,10 +4680,10 @@
         <v>122</v>
       </c>
       <c r="D21" s="8">
+        <v>0</v>
+      </c>
+      <c r="F21" s="8">
         <v>0.01</v>
-      </c>
-      <c r="F21" s="8">
-        <v>0.06</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -4691,10 +4691,10 @@
         <v>123</v>
       </c>
       <c r="D22" s="8">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="F22" s="8">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
@@ -4702,10 +4702,10 @@
         <v>124</v>
       </c>
       <c r="D23" s="8">
-        <v>0.03</v>
+        <v>0.13</v>
       </c>
       <c r="F23" s="8">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>